<commit_message>
📊 Full pipeline output Tue Jun  2 09:00:45 UTC 2026
</commit_message>
<xml_diff>
--- a/output/intraday/riepilogo_intraday_2026-06-02.xlsx
+++ b/output/intraday/riepilogo_intraday_2026-06-02.xlsx
@@ -20,16 +20,13 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -40,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -48,21 +45,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -433,372 +421,372 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Ticker</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Gap%</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Market Cap</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Shs Float</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Shares Outstanding</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Change from Open</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Insider Ownership</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Institutional Ownership</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Short Float</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>VWAP_0930</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>Close</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>Volume</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>TimeHigh</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>TimeLow</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>OpenPM</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>HighPM</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>LowPM</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>ClosePM</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>VolumePM</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>TimePMH</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>High_1m</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>Low_1m</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>Volume_1m</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>Close_1m</t>
         </is>
       </c>
-      <c r="AC1" s="1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>High_5m</t>
         </is>
       </c>
-      <c r="AD1" s="1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>Low_5m</t>
         </is>
       </c>
-      <c r="AE1" s="1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>Volume_5m</t>
         </is>
       </c>
-      <c r="AF1" s="1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>Close_5m</t>
         </is>
       </c>
-      <c r="AG1" s="1" t="inlineStr">
+      <c r="AG1" t="inlineStr">
         <is>
           <t>High_15m</t>
         </is>
       </c>
-      <c r="AH1" s="1" t="inlineStr">
+      <c r="AH1" t="inlineStr">
         <is>
           <t>Low_15m</t>
         </is>
       </c>
-      <c r="AI1" s="1" t="inlineStr">
+      <c r="AI1" t="inlineStr">
         <is>
           <t>Volume_15m</t>
         </is>
       </c>
-      <c r="AJ1" s="1" t="inlineStr">
+      <c r="AJ1" t="inlineStr">
         <is>
           <t>Close_15m</t>
         </is>
       </c>
-      <c r="AK1" s="1" t="inlineStr">
+      <c r="AK1" t="inlineStr">
         <is>
           <t>High_30m</t>
         </is>
       </c>
-      <c r="AL1" s="1" t="inlineStr">
+      <c r="AL1" t="inlineStr">
         <is>
           <t>Low_30m</t>
         </is>
       </c>
-      <c r="AM1" s="1" t="inlineStr">
+      <c r="AM1" t="inlineStr">
         <is>
           <t>Volume_30m</t>
         </is>
       </c>
-      <c r="AN1" s="1" t="inlineStr">
+      <c r="AN1" t="inlineStr">
         <is>
           <t>Close_30m</t>
         </is>
       </c>
-      <c r="AO1" s="1" t="inlineStr">
+      <c r="AO1" t="inlineStr">
         <is>
           <t>High_45m</t>
         </is>
       </c>
-      <c r="AP1" s="1" t="inlineStr">
+      <c r="AP1" t="inlineStr">
         <is>
           <t>Low_45m</t>
         </is>
       </c>
-      <c r="AQ1" s="1" t="inlineStr">
+      <c r="AQ1" t="inlineStr">
         <is>
           <t>Volume_45m</t>
         </is>
       </c>
-      <c r="AR1" s="1" t="inlineStr">
+      <c r="AR1" t="inlineStr">
         <is>
           <t>Close_45m</t>
         </is>
       </c>
-      <c r="AS1" s="1" t="inlineStr">
+      <c r="AS1" t="inlineStr">
         <is>
           <t>High_60m</t>
         </is>
       </c>
-      <c r="AT1" s="1" t="inlineStr">
+      <c r="AT1" t="inlineStr">
         <is>
           <t>Low_60m</t>
         </is>
       </c>
-      <c r="AU1" s="1" t="inlineStr">
+      <c r="AU1" t="inlineStr">
         <is>
           <t>Volume_60m</t>
         </is>
       </c>
-      <c r="AV1" s="1" t="inlineStr">
+      <c r="AV1" t="inlineStr">
         <is>
           <t>Close_60m</t>
         </is>
       </c>
-      <c r="AW1" s="1" t="inlineStr">
+      <c r="AW1" t="inlineStr">
         <is>
           <t>High_90m</t>
         </is>
       </c>
-      <c r="AX1" s="1" t="inlineStr">
+      <c r="AX1" t="inlineStr">
         <is>
           <t>Low_90m</t>
         </is>
       </c>
-      <c r="AY1" s="1" t="inlineStr">
+      <c r="AY1" t="inlineStr">
         <is>
           <t>Volume_90m</t>
         </is>
       </c>
-      <c r="AZ1" s="1" t="inlineStr">
+      <c r="AZ1" t="inlineStr">
         <is>
           <t>Close_90m</t>
         </is>
       </c>
-      <c r="BA1" s="1" t="inlineStr">
+      <c r="BA1" t="inlineStr">
         <is>
           <t>High_120m</t>
         </is>
       </c>
-      <c r="BB1" s="1" t="inlineStr">
+      <c r="BB1" t="inlineStr">
         <is>
           <t>Low_120m</t>
         </is>
       </c>
-      <c r="BC1" s="1" t="inlineStr">
+      <c r="BC1" t="inlineStr">
         <is>
           <t>Volume_120m</t>
         </is>
       </c>
-      <c r="BD1" s="1" t="inlineStr">
+      <c r="BD1" t="inlineStr">
         <is>
           <t>Close_120m</t>
         </is>
       </c>
-      <c r="BE1" s="1" t="inlineStr">
+      <c r="BE1" t="inlineStr">
         <is>
           <t>High_240m</t>
         </is>
       </c>
-      <c r="BF1" s="1" t="inlineStr">
+      <c r="BF1" t="inlineStr">
         <is>
           <t>Low_240m</t>
         </is>
       </c>
-      <c r="BG1" s="1" t="inlineStr">
+      <c r="BG1" t="inlineStr">
         <is>
           <t>Volume_240m</t>
         </is>
       </c>
-      <c r="BH1" s="1" t="inlineStr">
+      <c r="BH1" t="inlineStr">
         <is>
           <t>Close_240m</t>
         </is>
       </c>
-      <c r="BI1" s="1" t="inlineStr">
+      <c r="BI1" t="inlineStr">
         <is>
           <t>High_5_15m</t>
         </is>
       </c>
-      <c r="BJ1" s="1" t="inlineStr">
+      <c r="BJ1" t="inlineStr">
         <is>
           <t>Low_5_15m</t>
         </is>
       </c>
-      <c r="BK1" s="1" t="inlineStr">
+      <c r="BK1" t="inlineStr">
         <is>
           <t>High_15_30m</t>
         </is>
       </c>
-      <c r="BL1" s="1" t="inlineStr">
+      <c r="BL1" t="inlineStr">
         <is>
           <t>Low_15_30m</t>
         </is>
       </c>
-      <c r="BM1" s="1" t="inlineStr">
+      <c r="BM1" t="inlineStr">
         <is>
           <t>High_30_45m</t>
         </is>
       </c>
-      <c r="BN1" s="1" t="inlineStr">
+      <c r="BN1" t="inlineStr">
         <is>
           <t>Low_30_45m</t>
         </is>
       </c>
-      <c r="BO1" s="1" t="inlineStr">
+      <c r="BO1" t="inlineStr">
         <is>
           <t>High_45_60m</t>
         </is>
       </c>
-      <c r="BP1" s="1" t="inlineStr">
+      <c r="BP1" t="inlineStr">
         <is>
           <t>Low_45_60m</t>
         </is>
       </c>
-      <c r="BQ1" s="1" t="inlineStr">
+      <c r="BQ1" t="inlineStr">
         <is>
           <t>High_60_90m</t>
         </is>
       </c>
-      <c r="BR1" s="1" t="inlineStr">
+      <c r="BR1" t="inlineStr">
         <is>
           <t>Low_60_90m</t>
         </is>
       </c>
-      <c r="BS1" s="1" t="inlineStr">
+      <c r="BS1" t="inlineStr">
         <is>
           <t>High_90_120m</t>
         </is>
       </c>
-      <c r="BT1" s="1" t="inlineStr">
+      <c r="BT1" t="inlineStr">
         <is>
           <t>Low_90_120m</t>
         </is>
       </c>
-      <c r="BU1" s="1" t="inlineStr">
+      <c r="BU1" t="inlineStr">
         <is>
           <t>High_120_240m</t>
         </is>
       </c>
-      <c r="BV1" s="1" t="inlineStr">
+      <c r="BV1" t="inlineStr">
         <is>
           <t>Low_120_240m</t>
         </is>
@@ -810,7 +798,7 @@
           <t>ABTS</t>
         </is>
       </c>
-      <c r="B2" s="2" t="n">
+      <c r="B2" s="1" t="n">
         <v>46174</v>
       </c>
       <c r="C2" t="n">
@@ -1044,7 +1032,7 @@
           <t>ANY</t>
         </is>
       </c>
-      <c r="B3" s="2" t="n">
+      <c r="B3" s="1" t="n">
         <v>46174</v>
       </c>
       <c r="C3" t="n">
@@ -1278,7 +1266,7 @@
           <t>CRE</t>
         </is>
       </c>
-      <c r="B4" s="2" t="n">
+      <c r="B4" s="1" t="n">
         <v>46174</v>
       </c>
       <c r="C4" t="n">
@@ -1512,7 +1500,7 @@
           <t>GNTA</t>
         </is>
       </c>
-      <c r="B5" s="2" t="n">
+      <c r="B5" s="1" t="n">
         <v>46174</v>
       </c>
       <c r="C5" t="n">
@@ -1587,7 +1575,7 @@
         <v>1.86</v>
       </c>
       <c r="Z5" t="n">
-        <v>1.71</v>
+        <v>1.72</v>
       </c>
       <c r="AA5" t="n">
         <v>298695</v>
@@ -1599,7 +1587,7 @@
         <v>2.19</v>
       </c>
       <c r="AD5" t="n">
-        <v>1.71</v>
+        <v>1.72</v>
       </c>
       <c r="AE5" t="n">
         <v>1035030</v>
@@ -1611,7 +1599,7 @@
         <v>2.3</v>
       </c>
       <c r="AH5" t="n">
-        <v>1.71</v>
+        <v>1.72</v>
       </c>
       <c r="AI5" t="n">
         <v>4094473</v>
@@ -1623,7 +1611,7 @@
         <v>2.3</v>
       </c>
       <c r="AL5" t="n">
-        <v>1.71</v>
+        <v>1.72</v>
       </c>
       <c r="AM5" t="n">
         <v>5748528</v>
@@ -1635,7 +1623,7 @@
         <v>2.3</v>
       </c>
       <c r="AP5" t="n">
-        <v>1.71</v>
+        <v>1.72</v>
       </c>
       <c r="AQ5" t="n">
         <v>6895557</v>
@@ -1740,7 +1728,7 @@
           <t>HKIT</t>
         </is>
       </c>
-      <c r="B6" s="2" t="n">
+      <c r="B6" s="1" t="n">
         <v>46174</v>
       </c>
       <c r="C6" t="n">
@@ -1974,7 +1962,7 @@
           <t>MASK</t>
         </is>
       </c>
-      <c r="B7" s="2" t="n">
+      <c r="B7" s="1" t="n">
         <v>46174</v>
       </c>
       <c r="C7" t="n">
@@ -2208,7 +2196,7 @@
           <t>NAMM</t>
         </is>
       </c>
-      <c r="B8" s="2" t="n">
+      <c r="B8" s="1" t="n">
         <v>46174</v>
       </c>
       <c r="C8" t="n">
@@ -2442,7 +2430,7 @@
           <t>TGHL</t>
         </is>
       </c>
-      <c r="B9" s="2" t="n">
+      <c r="B9" s="1" t="n">
         <v>46174</v>
       </c>
       <c r="C9" t="n">

</xml_diff>